<commit_message>
NTRAD addition of Estate and PTE Composite, update of Multibill and IWP23SelIDE
</commit_message>
<xml_diff>
--- a/KatalonData/MultibillTestData/MultibillCCData.xlsx
+++ b/KatalonData/MultibillTestData/MultibillCCData.xlsx
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1028" uniqueCount="292">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1068" uniqueCount="312">
   <si>
     <t>Result</t>
   </si>
@@ -920,6 +920,66 @@
   </si>
   <si>
     <t>Thu Mar 12 10:35:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 12:55:08 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 13:24:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 14:44:46 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 14:45:14 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 14:45:46 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 14:50:36 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 14:57:24 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:02:06 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:05:06 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:07:30 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:08:12 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:11:05 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:16:19 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:20:55 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:24:04 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:25:44 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:26:51 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:35:20 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:35:55 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri Jul 17 15:36:56 EDT 2026</t>
   </si>
 </sst>
 </file>
@@ -1349,7 +1409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AA2"/>
+  <dimension ref="A1:Z2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:26" x14ac:dyDescent="0.4">
@@ -1512,7 +1572,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A8BF27D-9E5B-43D3-A8C6-55BD0B2E602C}">
-  <dimension ref="A1:G2"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="24.4609375" collapsed="true"/>
@@ -1553,7 +1613,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71D7CF63-52CE-45A5-AAAD-49E5406A5D05}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="6" max="6" bestFit="true" customWidth="true" width="12.4609375" collapsed="true"/>
@@ -1593,11 +1653,11 @@
       </c>
     </row>
     <row ht="43.75" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>280</v>
+      <c r="B2" t="s" s="0">
+        <v>299</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1623,31 +1683,31 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>109</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="0">
         <v>698</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" t="s" s="0">
         <v>89</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" t="s" s="0">
         <v>90</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="0">
         <v>0</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="0">
         <v>0</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="0">
         <v>697</v>
       </c>
     </row>
@@ -1658,7 +1718,7 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{176BCD28-A901-4577-AC2B-4D8F84F5F4AB}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
@@ -1694,11 +1754,11 @@
       </c>
     </row>
     <row ht="43.75" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>282</v>
+      <c r="B2" t="s" s="0">
+        <v>301</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1730,7 +1790,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBAB8D87-1612-4A54-9789-20EBA3899496}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:5" x14ac:dyDescent="0.4">
@@ -1751,11 +1811,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>288</v>
+      <c r="B2" t="s" s="0">
+        <v>309</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1766,16 +1826,16 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B3" t="s">
-        <v>289</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="B3" t="s" s="0">
+        <v>310</v>
+      </c>
+      <c r="D3" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>85</v>
       </c>
     </row>
@@ -1786,7 +1846,7 @@
 
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C795593-D462-4484-9AA4-88FCDAFE3571}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
@@ -1822,11 +1882,11 @@
       </c>
     </row>
     <row ht="43.75" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>281</v>
+      <c r="B2" t="s" s="0">
+        <v>300</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1852,31 +1912,31 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>110</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>93</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" t="s" s="0">
         <v>94</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" t="s" s="0">
         <v>95</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="0">
         <v>0</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="0">
         <v>98</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="0">
         <v>789654</v>
       </c>
     </row>
@@ -1887,7 +1947,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{922E2DF4-99DD-461B-8823-21A4F73EC265}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
@@ -1923,11 +1983,11 @@
       </c>
     </row>
     <row ht="58.3" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>283</v>
+      <c r="B2" t="s" s="0">
+        <v>302</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -1959,7 +2019,7 @@
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D2F5DCD-3C8F-4880-BB50-8902A2B8FCEA}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="6" max="6" bestFit="true" customWidth="true" width="16.4609375" collapsed="true"/>
@@ -2000,11 +2060,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>287</v>
+      <c r="B2" t="s" s="0">
+        <v>307</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2036,7 +2096,7 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97872C09-914A-48DE-8F4E-FDB918E9AE67}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" bestFit="true" customWidth="true" width="5.61328125" collapsed="true"/>
@@ -2079,11 +2139,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>278</v>
+      <c r="B2" t="s" s="0">
+        <v>298</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2109,16 +2169,16 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>108</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>46</v>
       </c>
     </row>
@@ -2129,7 +2189,7 @@
 
 <file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EBC5830D-66D0-4550-8001-686B3F1A766F}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
@@ -2165,11 +2225,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>284</v>
+      <c r="B2" t="s" s="0">
+        <v>304</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2195,16 +2255,16 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>115</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>57</v>
       </c>
     </row>
@@ -2215,7 +2275,7 @@
 
 <file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0BA84A4D-C922-4030-9CED-DABBEF75479D}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
@@ -2251,11 +2311,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>286</v>
+      <c r="B2" t="s" s="0">
+        <v>306</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2281,16 +2341,16 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>112</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>98</v>
       </c>
     </row>
@@ -2301,7 +2361,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A683BE9-6249-421D-92CB-328DFD4DF946}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="25.921875" collapsed="true"/>
@@ -2344,11 +2404,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>274</v>
+      <c r="B2" t="s" s="0">
+        <v>308</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2374,10 +2434,10 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>113</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -2409,7 +2469,7 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F12B0A87-644D-4675-93A2-DC39D9AADE64}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:10" x14ac:dyDescent="0.4">
@@ -2445,11 +2505,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>285</v>
+      <c r="B2" t="s" s="0">
+        <v>305</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2475,16 +2535,16 @@
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>111</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>57</v>
       </c>
     </row>
@@ -2495,7 +2555,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{051F4528-1B41-4D78-BCA4-48AC174370CB}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="25.921875" collapsed="true"/>
@@ -2534,11 +2594,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>276</v>
+      <c r="B2" t="s" s="0">
+        <v>297</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2579,7 +2639,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{320D1D33-46D9-47A1-8D21-2F325C6EB804}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="7" max="7" bestFit="true" customWidth="true" width="15.921875" collapsed="true"/>
@@ -2618,10 +2678,10 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" t="s" s="0">
         <v>119</v>
       </c>
       <c r="C2" s="1"/>
@@ -2659,7 +2719,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{869053C2-BECE-477A-A52F-F9A660E766F1}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="25.921875" collapsed="true"/>
@@ -2698,11 +2758,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>258</v>
+      <c r="B2" t="s" s="0">
+        <v>296</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2734,7 +2794,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB854B13-0493-48E8-AA80-CD6F2F5005DA}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" bestFit="true" customWidth="true" width="5.921875" collapsed="true"/>
@@ -2782,11 +2842,11 @@
       </c>
     </row>
     <row ht="29.15" r="2" spans="1:10" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>291</v>
+      <c r="B2" t="s" s="0">
+        <v>294</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -2818,7 +2878,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36947155-855C-418A-BB46-98E870DFBFDC}">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="2" max="2" bestFit="true" customWidth="true" width="25.61328125" collapsed="true"/>
@@ -2949,7 +3009,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E46036D-3E0A-4CA8-9437-AC70B02E484B}">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row ht="29.15" r="1" spans="1:15" x14ac:dyDescent="0.4">
@@ -2997,11 +3057,11 @@
       </c>
     </row>
     <row ht="113.15" r="2" spans="1:15" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>272</v>
+      <c r="B2" t="s" s="0">
+        <v>311</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -3048,7 +3108,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B0777A2-8D17-46EC-97AB-260FCB0FA79E}">
-  <dimension ref="A1:F3"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" bestFit="true" customWidth="true" width="5.61328125" collapsed="true"/>
@@ -3072,11 +3132,11 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+      <c r="A2" t="s" s="0">
         <v>56</v>
       </c>
-      <c r="B2" t="s">
-        <v>273</v>
+      <c r="B2" t="s" s="0">
+        <v>303</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
@@ -3087,16 +3147,16 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" t="s" s="0">
         <v>58</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" t="s" s="0">
         <v>114</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" t="s" s="0">
         <v>116</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" t="s" s="0">
         <v>85</v>
       </c>
     </row>

</xml_diff>